<commit_message>
fix: update main_rd PSF bundle path
</commit_message>
<xml_diff>
--- a/config/et_100_det_inputs_1h.xlsx
+++ b/config/et_100_det_inputs_1h.xlsx
@@ -1636,7 +1636,7 @@
       </c>
       <c r="C32" s="48" t="inlineStr">
         <is>
-          <t>241006/D280mm-focus</t>
+          <t>psf/et/241006/D280mm-focus</t>
         </is>
       </c>
       <c r="D32" s="54" t="n"/>
@@ -3999,6 +3999,14 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="41">
       <c r="A15" s="71" t="inlineStr">
         <is>
@@ -4030,12 +4038,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:B2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="200.85" customWidth="1" style="58" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="342.75" customHeight="1" s="41">
       <c r="B2" s="58" t="inlineStr">
         <is>

</xml_diff>